<commit_message>
Fixes Done, Except Settlement
</commit_message>
<xml_diff>
--- a/Encollect_Web_SCB_P3/Cypress/fixtures/Bulktrail.xlsx
+++ b/Encollect_Web_SCB_P3/Cypress/fixtures/Bulktrail.xlsx
@@ -451,7 +451,7 @@
         <v>1667</v>
       </c>
       <c r="B2" t="str">
-        <v>1660</v>
+        <v>10031</v>
       </c>
       <c r="C2" t="str">
         <v>Yes</v>
@@ -460,10 +460,10 @@
         <v>PTP</v>
       </c>
       <c r="E2" t="str">
-        <v>BOTP</v>
+        <v>PTP</v>
       </c>
       <c r="F2" t="str">
-        <v>2025-06-28</v>
+        <v>2027-06-28</v>
       </c>
       <c r="G2" t="str">
         <v>21524</v>

</xml_diff>

<commit_message>
Adding Nov Framework and Execution Completed For UAT
</commit_message>
<xml_diff>
--- a/Encollect_Web_SCB_P3/Cypress/fixtures/Bulktrail.xlsx
+++ b/Encollect_Web_SCB_P3/Cypress/fixtures/Bulktrail.xlsx
@@ -451,7 +451,7 @@
         <v>1667</v>
       </c>
       <c r="B2" t="str">
-        <v>10031</v>
+        <v>1660</v>
       </c>
       <c r="C2" t="str">
         <v>Yes</v>
@@ -460,10 +460,10 @@
         <v>PTP</v>
       </c>
       <c r="E2" t="str">
-        <v>PTP</v>
+        <v>BOTP</v>
       </c>
       <c r="F2" t="str">
-        <v>2027-06-28</v>
+        <v>2025-06-28</v>
       </c>
       <c r="G2" t="str">
         <v>21524</v>

</xml_diff>